<commit_message>
Fix margenes plantilla Excel
</commit_message>
<xml_diff>
--- a/ModuloWeb1/Plantillas/PlantillaOrdenes.xlsx
+++ b/ModuloWeb1/Plantillas/PlantillaOrdenes.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Asus\Desktop\milo\moduloweb-ordenes-compra\ModuloWeb1\Plantillas\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2738177A-CF18-4C46-9123-83C3D39A85A5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{88B60066-CF47-4742-87B3-3A83606C84E1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="2700" yWindow="2330" windowWidth="14400" windowHeight="7360" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
@@ -742,12 +742,58 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="165" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="169" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="169" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="3" fillId="0" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="3" fontId="8" fillId="2" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
     <xf numFmtId="0" fontId="6" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
@@ -757,58 +803,12 @@
     <xf numFmtId="0" fontId="3" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="3" fontId="8" fillId="2" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="169" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
-    <xf numFmtId="169" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="3" fillId="0" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1229,10 +1229,10 @@
       <c r="M1" s="1"/>
     </row>
     <row r="2" spans="2:14" ht="12.75" customHeight="1">
-      <c r="L2" s="85"/>
+      <c r="L2" s="54"/>
     </row>
     <row r="3" spans="2:14" ht="12.75" customHeight="1">
-      <c r="L3" s="86"/>
+      <c r="L3" s="55"/>
     </row>
     <row r="4" spans="2:14" ht="12.75" customHeight="1"/>
     <row r="5" spans="2:14" ht="12.5" customHeight="1">
@@ -1253,188 +1253,188 @@
     </row>
     <row r="7" spans="2:14" ht="6.75" customHeight="1"/>
     <row r="8" spans="2:14" ht="12.75" customHeight="1">
-      <c r="B8" s="54" t="str">
+      <c r="B8" s="83" t="str">
         <f>"Proveedor: " &amp; Instancia!L2</f>
         <v>Proveedor: ABB_COLOMBIA_LTDA</v>
       </c>
-      <c r="C8" s="55"/>
-      <c r="D8" s="55"/>
-      <c r="E8" s="55"/>
-      <c r="F8" s="55"/>
-      <c r="G8" s="56"/>
+      <c r="C8" s="84"/>
+      <c r="D8" s="84"/>
+      <c r="E8" s="84"/>
+      <c r="F8" s="84"/>
+      <c r="G8" s="85"/>
       <c r="H8" s="5"/>
-      <c r="J8" s="54" t="s">
+      <c r="J8" s="83" t="s">
         <v>0</v>
       </c>
-      <c r="K8" s="55"/>
-      <c r="L8" s="55"/>
-      <c r="M8" s="55"/>
-      <c r="N8" s="57"/>
+      <c r="K8" s="84"/>
+      <c r="L8" s="84"/>
+      <c r="M8" s="84"/>
+      <c r="N8" s="86"/>
     </row>
     <row r="9" spans="2:14" ht="12.75" customHeight="1">
-      <c r="B9" s="58" t="str">
+      <c r="B9" s="78" t="str">
         <f>"NIT/CC: " &amp; Instancia!M2</f>
         <v>NIT/CC: 901283882-1</v>
       </c>
-      <c r="C9" s="59"/>
-      <c r="D9" s="59"/>
-      <c r="E9" s="59"/>
-      <c r="F9" s="59"/>
-      <c r="G9" s="59"/>
-      <c r="H9" s="60"/>
-      <c r="J9" s="58" t="s">
+      <c r="C9" s="79"/>
+      <c r="D9" s="79"/>
+      <c r="E9" s="79"/>
+      <c r="F9" s="79"/>
+      <c r="G9" s="79"/>
+      <c r="H9" s="80"/>
+      <c r="J9" s="78" t="s">
         <v>1</v>
       </c>
-      <c r="K9" s="59"/>
-      <c r="L9" s="59"/>
-      <c r="M9" s="59"/>
-      <c r="N9" s="60"/>
+      <c r="K9" s="79"/>
+      <c r="L9" s="79"/>
+      <c r="M9" s="79"/>
+      <c r="N9" s="80"/>
     </row>
     <row r="10" spans="2:14" ht="12.75" customHeight="1">
-      <c r="B10" s="58" t="str">
+      <c r="B10" s="78" t="str">
         <f>"Ciudad: " &amp; Instancia!N2</f>
         <v>Ciudad: Bogotá</v>
       </c>
-      <c r="C10" s="59"/>
-      <c r="D10" s="59"/>
-      <c r="E10" s="59"/>
-      <c r="F10" s="59"/>
-      <c r="G10" s="59"/>
-      <c r="H10" s="60"/>
-      <c r="J10" s="58" t="s">
+      <c r="C10" s="79"/>
+      <c r="D10" s="79"/>
+      <c r="E10" s="79"/>
+      <c r="F10" s="79"/>
+      <c r="G10" s="79"/>
+      <c r="H10" s="80"/>
+      <c r="J10" s="78" t="s">
         <v>2</v>
       </c>
-      <c r="K10" s="59"/>
-      <c r="L10" s="59"/>
-      <c r="M10" s="59"/>
-      <c r="N10" s="60"/>
+      <c r="K10" s="79"/>
+      <c r="L10" s="79"/>
+      <c r="M10" s="79"/>
+      <c r="N10" s="80"/>
     </row>
     <row r="11" spans="2:14" ht="12.75" customHeight="1">
-      <c r="B11" s="58" t="str">
+      <c r="B11" s="78" t="str">
         <f>"Dirección: " &amp; Instancia!O2</f>
         <v>Dirección: CR 45 108 27 TO 1 P 12 (!) PARALELO 108</v>
       </c>
-      <c r="C11" s="59"/>
-      <c r="D11" s="59"/>
-      <c r="E11" s="59"/>
-      <c r="F11" s="59"/>
-      <c r="G11" s="59"/>
-      <c r="H11" s="60"/>
-      <c r="J11" s="58" t="s">
+      <c r="C11" s="79"/>
+      <c r="D11" s="79"/>
+      <c r="E11" s="79"/>
+      <c r="F11" s="79"/>
+      <c r="G11" s="79"/>
+      <c r="H11" s="80"/>
+      <c r="J11" s="78" t="s">
         <v>3</v>
       </c>
-      <c r="K11" s="59"/>
-      <c r="L11" s="59"/>
-      <c r="M11" s="59"/>
-      <c r="N11" s="60"/>
+      <c r="K11" s="79"/>
+      <c r="L11" s="79"/>
+      <c r="M11" s="79"/>
+      <c r="N11" s="80"/>
     </row>
     <row r="12" spans="2:14" ht="12.75" hidden="1" customHeight="1">
-      <c r="B12" s="58" t="s">
+      <c r="B12" s="78" t="s">
         <v>4</v>
       </c>
-      <c r="C12" s="59"/>
-      <c r="D12" s="59"/>
-      <c r="E12" s="59"/>
-      <c r="F12" s="59"/>
-      <c r="G12" s="59"/>
-      <c r="H12" s="60"/>
-      <c r="J12" s="58" t="s">
+      <c r="C12" s="79"/>
+      <c r="D12" s="79"/>
+      <c r="E12" s="79"/>
+      <c r="F12" s="79"/>
+      <c r="G12" s="79"/>
+      <c r="H12" s="80"/>
+      <c r="J12" s="78" t="s">
         <v>5</v>
       </c>
-      <c r="K12" s="59"/>
-      <c r="L12" s="61"/>
-      <c r="M12" s="62" t="s">
+      <c r="K12" s="79"/>
+      <c r="L12" s="81"/>
+      <c r="M12" s="82" t="s">
         <v>6</v>
       </c>
-      <c r="N12" s="60"/>
+      <c r="N12" s="80"/>
     </row>
     <row r="13" spans="2:14" ht="22.5" customHeight="1">
-      <c r="B13" s="63" t="str">
+      <c r="B13" s="67" t="str">
         <f>"Contacto: " &amp; Instancia!C2</f>
         <v>Contacto: DIEGO ZAPATA</v>
       </c>
-      <c r="C13" s="64"/>
-      <c r="D13" s="64"/>
-      <c r="E13" s="65"/>
-      <c r="F13" s="66"/>
-      <c r="G13" s="64"/>
-      <c r="H13" s="67"/>
-      <c r="J13" s="68" t="s">
+      <c r="C13" s="68"/>
+      <c r="D13" s="68"/>
+      <c r="E13" s="69"/>
+      <c r="F13" s="70"/>
+      <c r="G13" s="68"/>
+      <c r="H13" s="71"/>
+      <c r="J13" s="72" t="s">
         <v>7</v>
       </c>
-      <c r="K13" s="69"/>
-      <c r="L13" s="69"/>
-      <c r="M13" s="69"/>
-      <c r="N13" s="70"/>
+      <c r="K13" s="73"/>
+      <c r="L13" s="73"/>
+      <c r="M13" s="73"/>
+      <c r="N13" s="74"/>
     </row>
     <row r="14" spans="2:14" ht="12.75" customHeight="1">
-      <c r="B14" s="71" t="s">
+      <c r="B14" s="75" t="s">
         <v>8</v>
       </c>
-      <c r="C14" s="72"/>
-      <c r="D14" s="73"/>
-      <c r="E14" s="74" t="s">
+      <c r="C14" s="60"/>
+      <c r="D14" s="61"/>
+      <c r="E14" s="76" t="s">
         <v>9</v>
       </c>
-      <c r="F14" s="73"/>
-      <c r="G14" s="74" t="s">
+      <c r="F14" s="61"/>
+      <c r="G14" s="76" t="s">
         <v>10</v>
       </c>
-      <c r="H14" s="72"/>
-      <c r="I14" s="73"/>
-      <c r="J14" s="75" t="str">
+      <c r="H14" s="60"/>
+      <c r="I14" s="61"/>
+      <c r="J14" s="77" t="str">
         <f>"Entregar a Alterno: " &amp; Instancia!H2</f>
         <v>Entregar a Alterno: NA</v>
       </c>
-      <c r="K14" s="72"/>
-      <c r="L14" s="72"/>
-      <c r="M14" s="72"/>
-      <c r="N14" s="73"/>
+      <c r="K14" s="60"/>
+      <c r="L14" s="60"/>
+      <c r="M14" s="60"/>
+      <c r="N14" s="61"/>
     </row>
     <row r="15" spans="2:14" ht="12.75" customHeight="1">
-      <c r="B15" s="83">
+      <c r="B15" s="65">
         <f>Instancia!E2</f>
         <v>45875</v>
       </c>
-      <c r="C15" s="72"/>
-      <c r="D15" s="73"/>
-      <c r="E15" s="84" t="str">
+      <c r="C15" s="60"/>
+      <c r="D15" s="61"/>
+      <c r="E15" s="66" t="str">
         <f>Instancia!F2</f>
         <v>USD</v>
       </c>
-      <c r="F15" s="73"/>
-      <c r="G15" s="84" t="str">
+      <c r="F15" s="61"/>
+      <c r="G15" s="66" t="str">
         <f>Instancia!P2</f>
         <v>ANNI CARMONA</v>
       </c>
-      <c r="H15" s="72"/>
-      <c r="I15" s="73"/>
-      <c r="J15" s="79" t="str">
+      <c r="H15" s="60"/>
+      <c r="I15" s="61"/>
+      <c r="J15" s="59" t="str">
         <f>"Entregar a: " &amp; Instancia!G2</f>
         <v>Entregar a: SUPLINDUSTRA SAS</v>
       </c>
-      <c r="K15" s="72"/>
-      <c r="L15" s="72"/>
-      <c r="M15" s="72"/>
-      <c r="N15" s="73"/>
+      <c r="K15" s="60"/>
+      <c r="L15" s="60"/>
+      <c r="M15" s="60"/>
+      <c r="N15" s="61"/>
     </row>
     <row r="16" spans="2:14" ht="12.75" customHeight="1">
-      <c r="B16" s="80" t="str">
+      <c r="B16" s="62" t="str">
         <f>"Condiciones de pago: " &amp; Instancia!I2</f>
         <v>Condiciones de pago: CRÉDITO</v>
       </c>
-      <c r="C16" s="72"/>
-      <c r="D16" s="72"/>
-      <c r="E16" s="72"/>
-      <c r="F16" s="72"/>
-      <c r="G16" s="72"/>
-      <c r="H16" s="72"/>
-      <c r="I16" s="72"/>
-      <c r="J16" s="72"/>
-      <c r="K16" s="72"/>
-      <c r="L16" s="72"/>
-      <c r="M16" s="72"/>
-      <c r="N16" s="73"/>
+      <c r="C16" s="60"/>
+      <c r="D16" s="60"/>
+      <c r="E16" s="60"/>
+      <c r="F16" s="60"/>
+      <c r="G16" s="60"/>
+      <c r="H16" s="60"/>
+      <c r="I16" s="60"/>
+      <c r="J16" s="60"/>
+      <c r="K16" s="60"/>
+      <c r="L16" s="60"/>
+      <c r="M16" s="60"/>
+      <c r="N16" s="61"/>
     </row>
     <row r="17" spans="2:15" ht="22.5" customHeight="1"/>
     <row r="18" spans="2:15" ht="24.75" customHeight="1">
@@ -1615,32 +1615,32 @@
     <row r="28" spans="2:15" ht="112.5" hidden="1" customHeight="1">
       <c r="B28" s="28"/>
       <c r="C28" s="29"/>
-      <c r="D28" s="81"/>
-      <c r="E28" s="82"/>
-      <c r="F28" s="81"/>
-      <c r="G28" s="82"/>
-      <c r="H28" s="82"/>
-      <c r="I28" s="81"/>
-      <c r="J28" s="81"/>
+      <c r="D28" s="63"/>
+      <c r="E28" s="64"/>
+      <c r="F28" s="63"/>
+      <c r="G28" s="64"/>
+      <c r="H28" s="64"/>
+      <c r="I28" s="63"/>
+      <c r="J28" s="63"/>
       <c r="K28" s="31"/>
-      <c r="L28" s="76"/>
+      <c r="L28" s="56"/>
       <c r="M28" s="26"/>
-      <c r="N28" s="78"/>
+      <c r="N28" s="58"/>
     </row>
     <row r="29" spans="2:15" ht="112.5" hidden="1" customHeight="1">
       <c r="B29" s="28"/>
       <c r="C29" s="29"/>
-      <c r="D29" s="77"/>
-      <c r="E29" s="77"/>
-      <c r="F29" s="77"/>
-      <c r="G29" s="77"/>
-      <c r="H29" s="77"/>
-      <c r="I29" s="77"/>
-      <c r="J29" s="77"/>
+      <c r="D29" s="57"/>
+      <c r="E29" s="57"/>
+      <c r="F29" s="57"/>
+      <c r="G29" s="57"/>
+      <c r="H29" s="57"/>
+      <c r="I29" s="57"/>
+      <c r="J29" s="57"/>
       <c r="K29" s="31"/>
-      <c r="L29" s="77"/>
+      <c r="L29" s="57"/>
       <c r="M29" s="26"/>
-      <c r="N29" s="77"/>
+      <c r="N29" s="57"/>
     </row>
     <row r="30" spans="2:15" ht="112.5" customHeight="1">
       <c r="B30" s="28"/>
@@ -2865,6 +2865,24 @@
     <row r="1000" ht="12.75" customHeight="1"/>
   </sheetData>
   <mergeCells count="32">
+    <mergeCell ref="B8:G8"/>
+    <mergeCell ref="J8:N8"/>
+    <mergeCell ref="B9:H9"/>
+    <mergeCell ref="J9:N9"/>
+    <mergeCell ref="B10:H10"/>
+    <mergeCell ref="J10:N10"/>
+    <mergeCell ref="J11:N11"/>
+    <mergeCell ref="B11:H11"/>
+    <mergeCell ref="B12:H12"/>
+    <mergeCell ref="J12:L12"/>
+    <mergeCell ref="M12:N12"/>
+    <mergeCell ref="B13:E13"/>
+    <mergeCell ref="F13:H13"/>
+    <mergeCell ref="J13:N13"/>
+    <mergeCell ref="B14:D14"/>
+    <mergeCell ref="E14:F14"/>
+    <mergeCell ref="G14:I14"/>
+    <mergeCell ref="J14:N14"/>
     <mergeCell ref="L28:L29"/>
     <mergeCell ref="N28:N29"/>
     <mergeCell ref="J15:N15"/>
@@ -2879,29 +2897,11 @@
     <mergeCell ref="G15:I15"/>
     <mergeCell ref="I28:I29"/>
     <mergeCell ref="J28:J29"/>
-    <mergeCell ref="B13:E13"/>
-    <mergeCell ref="F13:H13"/>
-    <mergeCell ref="J13:N13"/>
-    <mergeCell ref="B14:D14"/>
-    <mergeCell ref="E14:F14"/>
-    <mergeCell ref="G14:I14"/>
-    <mergeCell ref="J14:N14"/>
-    <mergeCell ref="J11:N11"/>
-    <mergeCell ref="B11:H11"/>
-    <mergeCell ref="B12:H12"/>
-    <mergeCell ref="J12:L12"/>
-    <mergeCell ref="M12:N12"/>
-    <mergeCell ref="B8:G8"/>
-    <mergeCell ref="J8:N8"/>
-    <mergeCell ref="B9:H9"/>
-    <mergeCell ref="J9:N9"/>
-    <mergeCell ref="B10:H10"/>
-    <mergeCell ref="J10:N10"/>
   </mergeCells>
   <printOptions horizontalCentered="1"/>
-  <pageMargins left="0" right="0" top="0" bottom="0" header="0" footer="0"/>
-  <pageSetup paperSize="9" orientation="landscape"/>
-  <drawing r:id="rId1"/>
+  <pageMargins left="0.39370078740157483" right="0.39370078740157483" top="0.39370078740157483" bottom="0.39370078740157483" header="0.31496062992125984" footer="0.31496062992125984"/>
+  <pageSetup paperSize="9" scale="72" orientation="landscape" r:id="rId1"/>
+  <drawing r:id="rId2"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
Actualizar orden columnas y plantilla
</commit_message>
<xml_diff>
--- a/ModuloWeb1/Plantillas/PlantillaOrdenes.xlsx
+++ b/ModuloWeb1/Plantillas/PlantillaOrdenes.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Asus\Desktop\milo\moduloweb-ordenes-compra\ModuloWeb1\Plantillas\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{88B60066-CF47-4742-87B3-3A83606C84E1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{086B9B91-C8D3-4E46-AAC5-F36A31431B11}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2700" yWindow="2330" windowWidth="14400" windowHeight="7360" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
@@ -164,15 +164,9 @@
     <t>Item</t>
   </si>
   <si>
-    <t>Catalogo</t>
-  </si>
-  <si>
     <t>Modelo</t>
   </si>
   <si>
-    <t>Descripcion</t>
-  </si>
-  <si>
     <t>F. Entrega</t>
   </si>
   <si>
@@ -255,6 +249,12 @@
   </si>
   <si>
     <t>CRÉDITO</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Descripcion </t>
+  </si>
+  <si>
+    <t>N° Catálogo</t>
   </si>
 </sst>
 </file>
@@ -269,7 +269,7 @@
     <numFmt numFmtId="168" formatCode="_(&quot;$&quot;* #,##0.00_);_(&quot;$&quot;* \(#,##0.00\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
     <numFmt numFmtId="169" formatCode="_(&quot;$&quot;* #,##0_);_(&quot;$&quot;* \(#,##0\);_(&quot;$&quot;* &quot;-&quot;_);_(@_)"/>
   </numFmts>
-  <fonts count="12">
+  <fonts count="13">
     <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
@@ -336,6 +336,13 @@
       <sz val="12"/>
       <color rgb="FF202124"/>
       <name val="Docs-Roboto"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="5">
@@ -599,7 +606,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="87">
+  <cellXfs count="89">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="164" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
@@ -744,56 +751,12 @@
     <xf numFmtId="165" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="169" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
-    <xf numFmtId="169" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="3" fillId="0" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="3" fontId="8" fillId="2" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="6" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
@@ -803,12 +766,62 @@
     <xf numFmtId="0" fontId="3" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="3" fontId="8" fillId="2" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="169" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="169" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="3" fillId="0" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1212,7 +1225,7 @@
     <col min="1" max="1" width="2.7265625" customWidth="1"/>
     <col min="2" max="3" width="5" customWidth="1"/>
     <col min="4" max="4" width="13.6328125" customWidth="1"/>
-    <col min="5" max="5" width="32.7265625" customWidth="1"/>
+    <col min="5" max="5" width="38.1796875" customWidth="1"/>
     <col min="6" max="6" width="18" customWidth="1"/>
     <col min="7" max="7" width="25.453125" customWidth="1"/>
     <col min="8" max="8" width="19" customWidth="1"/>
@@ -1253,188 +1266,188 @@
     </row>
     <row r="7" spans="2:14" ht="6.75" customHeight="1"/>
     <row r="8" spans="2:14" ht="12.75" customHeight="1">
-      <c r="B8" s="83" t="str">
+      <c r="B8" s="56" t="str">
         <f>"Proveedor: " &amp; Instancia!L2</f>
         <v>Proveedor: ABB_COLOMBIA_LTDA</v>
       </c>
-      <c r="C8" s="84"/>
-      <c r="D8" s="84"/>
-      <c r="E8" s="84"/>
-      <c r="F8" s="84"/>
-      <c r="G8" s="85"/>
+      <c r="C8" s="57"/>
+      <c r="D8" s="57"/>
+      <c r="E8" s="57"/>
+      <c r="F8" s="57"/>
+      <c r="G8" s="58"/>
       <c r="H8" s="5"/>
-      <c r="J8" s="83" t="s">
+      <c r="J8" s="56" t="s">
         <v>0</v>
       </c>
-      <c r="K8" s="84"/>
-      <c r="L8" s="84"/>
-      <c r="M8" s="84"/>
-      <c r="N8" s="86"/>
+      <c r="K8" s="57"/>
+      <c r="L8" s="57"/>
+      <c r="M8" s="57"/>
+      <c r="N8" s="59"/>
     </row>
     <row r="9" spans="2:14" ht="12.75" customHeight="1">
-      <c r="B9" s="78" t="str">
+      <c r="B9" s="60" t="str">
         <f>"NIT/CC: " &amp; Instancia!M2</f>
         <v>NIT/CC: 901283882-1</v>
       </c>
-      <c r="C9" s="79"/>
-      <c r="D9" s="79"/>
-      <c r="E9" s="79"/>
-      <c r="F9" s="79"/>
-      <c r="G9" s="79"/>
-      <c r="H9" s="80"/>
-      <c r="J9" s="78" t="s">
+      <c r="C9" s="61"/>
+      <c r="D9" s="61"/>
+      <c r="E9" s="61"/>
+      <c r="F9" s="61"/>
+      <c r="G9" s="61"/>
+      <c r="H9" s="62"/>
+      <c r="J9" s="60" t="s">
         <v>1</v>
       </c>
-      <c r="K9" s="79"/>
-      <c r="L9" s="79"/>
-      <c r="M9" s="79"/>
-      <c r="N9" s="80"/>
+      <c r="K9" s="61"/>
+      <c r="L9" s="61"/>
+      <c r="M9" s="61"/>
+      <c r="N9" s="62"/>
     </row>
     <row r="10" spans="2:14" ht="12.75" customHeight="1">
-      <c r="B10" s="78" t="str">
+      <c r="B10" s="60" t="str">
         <f>"Ciudad: " &amp; Instancia!N2</f>
         <v>Ciudad: Bogotá</v>
       </c>
-      <c r="C10" s="79"/>
-      <c r="D10" s="79"/>
-      <c r="E10" s="79"/>
-      <c r="F10" s="79"/>
-      <c r="G10" s="79"/>
-      <c r="H10" s="80"/>
-      <c r="J10" s="78" t="s">
+      <c r="C10" s="61"/>
+      <c r="D10" s="61"/>
+      <c r="E10" s="61"/>
+      <c r="F10" s="61"/>
+      <c r="G10" s="61"/>
+      <c r="H10" s="62"/>
+      <c r="J10" s="60" t="s">
         <v>2</v>
       </c>
-      <c r="K10" s="79"/>
-      <c r="L10" s="79"/>
-      <c r="M10" s="79"/>
-      <c r="N10" s="80"/>
+      <c r="K10" s="61"/>
+      <c r="L10" s="61"/>
+      <c r="M10" s="61"/>
+      <c r="N10" s="62"/>
     </row>
     <row r="11" spans="2:14" ht="12.75" customHeight="1">
-      <c r="B11" s="78" t="str">
+      <c r="B11" s="60" t="str">
         <f>"Dirección: " &amp; Instancia!O2</f>
         <v>Dirección: CR 45 108 27 TO 1 P 12 (!) PARALELO 108</v>
       </c>
-      <c r="C11" s="79"/>
-      <c r="D11" s="79"/>
-      <c r="E11" s="79"/>
-      <c r="F11" s="79"/>
-      <c r="G11" s="79"/>
-      <c r="H11" s="80"/>
-      <c r="J11" s="78" t="s">
+      <c r="C11" s="61"/>
+      <c r="D11" s="61"/>
+      <c r="E11" s="61"/>
+      <c r="F11" s="61"/>
+      <c r="G11" s="61"/>
+      <c r="H11" s="62"/>
+      <c r="J11" s="60" t="s">
         <v>3</v>
       </c>
-      <c r="K11" s="79"/>
-      <c r="L11" s="79"/>
-      <c r="M11" s="79"/>
-      <c r="N11" s="80"/>
+      <c r="K11" s="61"/>
+      <c r="L11" s="61"/>
+      <c r="M11" s="61"/>
+      <c r="N11" s="62"/>
     </row>
     <row r="12" spans="2:14" ht="12.75" hidden="1" customHeight="1">
-      <c r="B12" s="78" t="s">
+      <c r="B12" s="60" t="s">
         <v>4</v>
       </c>
-      <c r="C12" s="79"/>
-      <c r="D12" s="79"/>
-      <c r="E12" s="79"/>
-      <c r="F12" s="79"/>
-      <c r="G12" s="79"/>
-      <c r="H12" s="80"/>
-      <c r="J12" s="78" t="s">
+      <c r="C12" s="61"/>
+      <c r="D12" s="61"/>
+      <c r="E12" s="61"/>
+      <c r="F12" s="61"/>
+      <c r="G12" s="61"/>
+      <c r="H12" s="62"/>
+      <c r="J12" s="60" t="s">
         <v>5</v>
       </c>
-      <c r="K12" s="79"/>
-      <c r="L12" s="81"/>
-      <c r="M12" s="82" t="s">
+      <c r="K12" s="61"/>
+      <c r="L12" s="63"/>
+      <c r="M12" s="64" t="s">
         <v>6</v>
       </c>
-      <c r="N12" s="80"/>
+      <c r="N12" s="62"/>
     </row>
     <row r="13" spans="2:14" ht="22.5" customHeight="1">
-      <c r="B13" s="67" t="str">
+      <c r="B13" s="65" t="str">
         <f>"Contacto: " &amp; Instancia!C2</f>
         <v>Contacto: DIEGO ZAPATA</v>
       </c>
-      <c r="C13" s="68"/>
-      <c r="D13" s="68"/>
-      <c r="E13" s="69"/>
-      <c r="F13" s="70"/>
-      <c r="G13" s="68"/>
-      <c r="H13" s="71"/>
-      <c r="J13" s="72" t="s">
+      <c r="C13" s="66"/>
+      <c r="D13" s="66"/>
+      <c r="E13" s="67"/>
+      <c r="F13" s="68"/>
+      <c r="G13" s="66"/>
+      <c r="H13" s="69"/>
+      <c r="J13" s="70" t="s">
         <v>7</v>
       </c>
-      <c r="K13" s="73"/>
-      <c r="L13" s="73"/>
-      <c r="M13" s="73"/>
-      <c r="N13" s="74"/>
+      <c r="K13" s="71"/>
+      <c r="L13" s="71"/>
+      <c r="M13" s="71"/>
+      <c r="N13" s="72"/>
     </row>
     <row r="14" spans="2:14" ht="12.75" customHeight="1">
-      <c r="B14" s="75" t="s">
+      <c r="B14" s="73" t="s">
         <v>8</v>
       </c>
-      <c r="C14" s="60"/>
-      <c r="D14" s="61"/>
+      <c r="C14" s="74"/>
+      <c r="D14" s="75"/>
       <c r="E14" s="76" t="s">
         <v>9</v>
       </c>
-      <c r="F14" s="61"/>
+      <c r="F14" s="75"/>
       <c r="G14" s="76" t="s">
         <v>10</v>
       </c>
-      <c r="H14" s="60"/>
-      <c r="I14" s="61"/>
+      <c r="H14" s="74"/>
+      <c r="I14" s="75"/>
       <c r="J14" s="77" t="str">
         <f>"Entregar a Alterno: " &amp; Instancia!H2</f>
         <v>Entregar a Alterno: NA</v>
       </c>
-      <c r="K14" s="60"/>
-      <c r="L14" s="60"/>
-      <c r="M14" s="60"/>
-      <c r="N14" s="61"/>
+      <c r="K14" s="74"/>
+      <c r="L14" s="74"/>
+      <c r="M14" s="74"/>
+      <c r="N14" s="75"/>
     </row>
     <row r="15" spans="2:14" ht="12.75" customHeight="1">
-      <c r="B15" s="65">
+      <c r="B15" s="85">
         <f>Instancia!E2</f>
         <v>45875</v>
       </c>
-      <c r="C15" s="60"/>
-      <c r="D15" s="61"/>
-      <c r="E15" s="66" t="str">
+      <c r="C15" s="74"/>
+      <c r="D15" s="75"/>
+      <c r="E15" s="86" t="str">
         <f>Instancia!F2</f>
         <v>USD</v>
       </c>
-      <c r="F15" s="61"/>
-      <c r="G15" s="66" t="str">
+      <c r="F15" s="75"/>
+      <c r="G15" s="86" t="str">
         <f>Instancia!P2</f>
         <v>ANNI CARMONA</v>
       </c>
-      <c r="H15" s="60"/>
-      <c r="I15" s="61"/>
-      <c r="J15" s="59" t="str">
+      <c r="H15" s="74"/>
+      <c r="I15" s="75"/>
+      <c r="J15" s="81" t="str">
         <f>"Entregar a: " &amp; Instancia!G2</f>
         <v>Entregar a: SUPLINDUSTRA SAS</v>
       </c>
-      <c r="K15" s="60"/>
-      <c r="L15" s="60"/>
-      <c r="M15" s="60"/>
-      <c r="N15" s="61"/>
+      <c r="K15" s="74"/>
+      <c r="L15" s="74"/>
+      <c r="M15" s="74"/>
+      <c r="N15" s="75"/>
     </row>
     <row r="16" spans="2:14" ht="12.75" customHeight="1">
-      <c r="B16" s="62" t="str">
+      <c r="B16" s="82" t="str">
         <f>"Condiciones de pago: " &amp; Instancia!I2</f>
         <v>Condiciones de pago: CRÉDITO</v>
       </c>
-      <c r="C16" s="60"/>
-      <c r="D16" s="60"/>
-      <c r="E16" s="60"/>
-      <c r="F16" s="60"/>
-      <c r="G16" s="60"/>
-      <c r="H16" s="60"/>
-      <c r="I16" s="60"/>
-      <c r="J16" s="60"/>
-      <c r="K16" s="60"/>
-      <c r="L16" s="60"/>
-      <c r="M16" s="60"/>
-      <c r="N16" s="61"/>
+      <c r="C16" s="74"/>
+      <c r="D16" s="74"/>
+      <c r="E16" s="74"/>
+      <c r="F16" s="74"/>
+      <c r="G16" s="74"/>
+      <c r="H16" s="74"/>
+      <c r="I16" s="74"/>
+      <c r="J16" s="74"/>
+      <c r="K16" s="74"/>
+      <c r="L16" s="74"/>
+      <c r="M16" s="74"/>
+      <c r="N16" s="75"/>
     </row>
     <row r="17" spans="2:15" ht="22.5" customHeight="1"/>
     <row r="18" spans="2:15" ht="24.75" customHeight="1">
@@ -1445,35 +1458,35 @@
       <c r="D18" s="7" t="s">
         <v>12</v>
       </c>
-      <c r="E18" s="7" t="s">
+      <c r="E18" s="87" t="s">
+        <v>42</v>
+      </c>
+      <c r="F18" s="7" t="s">
         <v>13</v>
       </c>
-      <c r="F18" s="7" t="s">
+      <c r="G18" s="87" t="s">
+        <v>43</v>
+      </c>
+      <c r="H18" s="7" t="s">
         <v>14</v>
       </c>
-      <c r="G18" s="7" t="s">
+      <c r="I18" s="7" t="s">
         <v>15</v>
       </c>
-      <c r="H18" s="7" t="s">
+      <c r="J18" s="7" t="s">
         <v>16</v>
       </c>
-      <c r="I18" s="7" t="s">
+      <c r="K18" s="7" t="s">
         <v>17</v>
       </c>
-      <c r="J18" s="7" t="s">
+      <c r="L18" s="7" t="s">
         <v>18</v>
       </c>
-      <c r="K18" s="7" t="s">
+      <c r="M18" s="7" t="s">
         <v>19</v>
       </c>
-      <c r="L18" s="7" t="s">
+      <c r="N18" s="7" t="s">
         <v>20</v>
-      </c>
-      <c r="M18" s="7" t="s">
-        <v>21</v>
-      </c>
-      <c r="N18" s="7" t="s">
-        <v>22</v>
       </c>
     </row>
     <row r="19" spans="2:15" ht="112.5" customHeight="1">
@@ -1482,7 +1495,7 @@
       <c r="D19" s="10"/>
       <c r="E19" s="11"/>
       <c r="F19" s="11"/>
-      <c r="G19" s="12"/>
+      <c r="G19" s="88"/>
       <c r="H19" s="13"/>
       <c r="I19" s="11"/>
       <c r="J19" s="11"/>
@@ -1615,32 +1628,32 @@
     <row r="28" spans="2:15" ht="112.5" hidden="1" customHeight="1">
       <c r="B28" s="28"/>
       <c r="C28" s="29"/>
-      <c r="D28" s="63"/>
-      <c r="E28" s="64"/>
-      <c r="F28" s="63"/>
-      <c r="G28" s="64"/>
-      <c r="H28" s="64"/>
-      <c r="I28" s="63"/>
-      <c r="J28" s="63"/>
+      <c r="D28" s="83"/>
+      <c r="E28" s="84"/>
+      <c r="F28" s="83"/>
+      <c r="G28" s="84"/>
+      <c r="H28" s="84"/>
+      <c r="I28" s="83"/>
+      <c r="J28" s="83"/>
       <c r="K28" s="31"/>
-      <c r="L28" s="56"/>
+      <c r="L28" s="78"/>
       <c r="M28" s="26"/>
-      <c r="N28" s="58"/>
+      <c r="N28" s="80"/>
     </row>
     <row r="29" spans="2:15" ht="112.5" hidden="1" customHeight="1">
       <c r="B29" s="28"/>
       <c r="C29" s="29"/>
-      <c r="D29" s="57"/>
-      <c r="E29" s="57"/>
-      <c r="F29" s="57"/>
-      <c r="G29" s="57"/>
-      <c r="H29" s="57"/>
-      <c r="I29" s="57"/>
-      <c r="J29" s="57"/>
+      <c r="D29" s="79"/>
+      <c r="E29" s="79"/>
+      <c r="F29" s="79"/>
+      <c r="G29" s="79"/>
+      <c r="H29" s="79"/>
+      <c r="I29" s="79"/>
+      <c r="J29" s="79"/>
       <c r="K29" s="31"/>
-      <c r="L29" s="57"/>
+      <c r="L29" s="79"/>
       <c r="M29" s="26"/>
-      <c r="N29" s="57"/>
+      <c r="N29" s="79"/>
     </row>
     <row r="30" spans="2:15" ht="112.5" customHeight="1">
       <c r="B30" s="28"/>
@@ -2865,24 +2878,6 @@
     <row r="1000" ht="12.75" customHeight="1"/>
   </sheetData>
   <mergeCells count="32">
-    <mergeCell ref="B8:G8"/>
-    <mergeCell ref="J8:N8"/>
-    <mergeCell ref="B9:H9"/>
-    <mergeCell ref="J9:N9"/>
-    <mergeCell ref="B10:H10"/>
-    <mergeCell ref="J10:N10"/>
-    <mergeCell ref="J11:N11"/>
-    <mergeCell ref="B11:H11"/>
-    <mergeCell ref="B12:H12"/>
-    <mergeCell ref="J12:L12"/>
-    <mergeCell ref="M12:N12"/>
-    <mergeCell ref="B13:E13"/>
-    <mergeCell ref="F13:H13"/>
-    <mergeCell ref="J13:N13"/>
-    <mergeCell ref="B14:D14"/>
-    <mergeCell ref="E14:F14"/>
-    <mergeCell ref="G14:I14"/>
-    <mergeCell ref="J14:N14"/>
     <mergeCell ref="L28:L29"/>
     <mergeCell ref="N28:N29"/>
     <mergeCell ref="J15:N15"/>
@@ -2897,6 +2892,24 @@
     <mergeCell ref="G15:I15"/>
     <mergeCell ref="I28:I29"/>
     <mergeCell ref="J28:J29"/>
+    <mergeCell ref="B13:E13"/>
+    <mergeCell ref="F13:H13"/>
+    <mergeCell ref="J13:N13"/>
+    <mergeCell ref="B14:D14"/>
+    <mergeCell ref="E14:F14"/>
+    <mergeCell ref="G14:I14"/>
+    <mergeCell ref="J14:N14"/>
+    <mergeCell ref="J11:N11"/>
+    <mergeCell ref="B11:H11"/>
+    <mergeCell ref="B12:H12"/>
+    <mergeCell ref="J12:L12"/>
+    <mergeCell ref="M12:N12"/>
+    <mergeCell ref="B8:G8"/>
+    <mergeCell ref="J8:N8"/>
+    <mergeCell ref="B9:H9"/>
+    <mergeCell ref="J9:N9"/>
+    <mergeCell ref="B10:H10"/>
+    <mergeCell ref="J10:N10"/>
   </mergeCells>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.39370078740157483" right="0.39370078740157483" top="0.39370078740157483" bottom="0.39370078740157483" header="0.31496062992125984" footer="0.31496062992125984"/>
@@ -2923,84 +2936,84 @@
   <sheetData>
     <row r="1" spans="2:26" ht="15" customHeight="1">
       <c r="B1" s="51" t="s">
+        <v>26</v>
+      </c>
+      <c r="C1" s="52" t="s">
+        <v>27</v>
+      </c>
+      <c r="D1" s="52" t="s">
         <v>28</v>
       </c>
-      <c r="C1" s="52" t="s">
+      <c r="E1" s="52" t="s">
         <v>29</v>
-      </c>
-      <c r="D1" s="52" t="s">
-        <v>30</v>
-      </c>
-      <c r="E1" s="52" t="s">
-        <v>31</v>
       </c>
       <c r="F1" s="51" t="s">
         <v>9</v>
       </c>
       <c r="G1" s="51" t="s">
+        <v>30</v>
+      </c>
+      <c r="H1" s="51" t="s">
+        <v>31</v>
+      </c>
+      <c r="I1" s="52" t="s">
         <v>32</v>
       </c>
-      <c r="H1" s="51" t="s">
+      <c r="J1" s="50" t="s">
         <v>33</v>
       </c>
-      <c r="I1" s="52" t="s">
+      <c r="K1" s="50" t="s">
         <v>34</v>
       </c>
-      <c r="J1" s="50" t="s">
+      <c r="L1" s="50" t="s">
         <v>35</v>
-      </c>
-      <c r="K1" s="50" t="s">
-        <v>36</v>
-      </c>
-      <c r="L1" s="50" t="s">
-        <v>37</v>
       </c>
     </row>
     <row r="2" spans="2:26" ht="15" customHeight="1">
       <c r="B2" s="50" t="s">
+        <v>36</v>
+      </c>
+      <c r="C2" s="50" t="s">
+        <v>37</v>
+      </c>
+      <c r="D2" s="50" t="s">
         <v>38</v>
-      </c>
-      <c r="C2" s="50" t="s">
-        <v>39</v>
-      </c>
-      <c r="D2" s="50" t="s">
-        <v>40</v>
       </c>
       <c r="E2" s="53">
         <v>45875</v>
       </c>
       <c r="F2" s="50" t="s">
+        <v>39</v>
+      </c>
+      <c r="G2" s="50" t="s">
+        <v>40</v>
+      </c>
+      <c r="H2" s="50" t="s">
+        <v>38</v>
+      </c>
+      <c r="I2" s="50" t="s">
         <v>41</v>
       </c>
-      <c r="G2" s="50" t="s">
-        <v>42</v>
-      </c>
-      <c r="H2" s="50" t="s">
-        <v>40</v>
-      </c>
-      <c r="I2" s="50" t="s">
-        <v>43</v>
-      </c>
       <c r="J2" s="50" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="K2" s="50" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="L2" s="50" t="s">
+        <v>22</v>
+      </c>
+      <c r="M2" s="50" t="s">
+        <v>23</v>
+      </c>
+      <c r="N2" s="50" t="s">
         <v>24</v>
       </c>
-      <c r="M2" s="50" t="s">
+      <c r="O2" s="50" t="s">
         <v>25</v>
       </c>
-      <c r="N2" s="50" t="s">
-        <v>26</v>
-      </c>
-      <c r="O2" s="50" t="s">
-        <v>27</v>
-      </c>
       <c r="P2" s="50" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="Q2" s="50"/>
       <c r="R2" s="50"/>

</xml_diff>